<commit_message>
harden template regeneration and preserve workbook fidelity
- keep rich text headers when migrating rows (rich_text=True)
- validate staged workbook before publishing; publish via ReplaceFileW on
  Windows to preserve destination ACL
- anchor sheet selection below frozen header rows to avoid double render
- drop no-op input-prompt validations on template columns
- regenerate gd templates, outputs and i18n files
</commit_message>
<xml_diff>
--- a/gd/excel/UIConfig.xlsx
+++ b/gd/excel/UIConfig.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -563,32 +563,117 @@
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Id
-int32</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Id
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF8A5A00"/>
+              <sz val="9"/>
+            </rPr>
+            <t>int32</t>
+          </r>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Layer
-UIConfigLayer</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Layer
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF64748B"/>
+              <sz val="9"/>
+            </rPr>
+            <t>UIConfigLayer</t>
+          </r>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>ResourceKey
-string</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">ResourceKey
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF64748B"/>
+              <sz val="9"/>
+            </rPr>
+            <t>string</t>
+          </r>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>BlocksRaycast
-bool</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">BlocksRaycast
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF64748B"/>
+              <sz val="9"/>
+            </rPr>
+            <t>bool</t>
+          </r>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Stack
-bool</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos"/>
+              <b val="1"/>
+              <color rgb="FF172033"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve">Stack
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Consolas"/>
+              <i val="1"/>
+              <color rgb="FF64748B"/>
+              <sz val="9"/>
+            </rPr>
+            <t>bool</t>
+          </r>
         </is>
       </c>
     </row>
@@ -716,6 +801,11 @@
       </c>
       <c r="E8" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>13003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>